<commit_message>
gu data 2025 reprocesssed changed yes/no is_hybrid in original data
</commit_message>
<xml_diff>
--- a/data/gu/original_data/gu Open APC Sweden 2025.xlsx
+++ b/data/gu/original_data/gu Open APC Sweden 2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xjopau\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/2021m30/R/repos/openapc-se/data/gu/original_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67AC3FDE-9FBE-4C97-B13A-7B77C20F541D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{008FAA51-B74F-BA4C-BB81-2040FBF56BEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="79080" yWindow="4020" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="article data" sheetId="1" r:id="rId1"/>
@@ -122,18 +122,12 @@
     <t>GU</t>
   </si>
   <si>
-    <t>NO</t>
-  </si>
-  <si>
     <t>MDPI</t>
   </si>
   <si>
     <t>10.1055/a-2761-5649</t>
   </si>
   <si>
-    <t>YES</t>
-  </si>
-  <si>
     <t>Thieme</t>
   </si>
   <si>
@@ -174,6 +168,12 @@
   </si>
   <si>
     <t>JAMA</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>FALSE</t>
   </si>
 </sst>
 </file>
@@ -522,22 +522,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K10"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.75" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.33203125" style="2" customWidth="1"/>
     <col min="5" max="6" width="10" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="3.375" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="11" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -572,7 +572,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>21</v>
       </c>
@@ -586,10 +586,10 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -603,16 +603,16 @@
         <v>35488</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>21</v>
       </c>
@@ -623,16 +623,16 @@
         <v>35680</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
@@ -643,19 +643,19 @@
         <v>28092</v>
       </c>
       <c r="D5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
@@ -666,16 +666,16 @@
         <v>28688</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
@@ -686,16 +686,16 @@
         <v>16294</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
@@ -706,16 +706,16 @@
         <v>25068</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -726,16 +726,16 @@
         <v>49474</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
@@ -746,13 +746,13 @@
         <v>35289</v>
       </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -772,21 +772,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E9D608-332C-6B41-B918-E0AD75CD6855}">
   <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="7.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="10.875" style="1"/>
+    <col min="9" max="10" width="7.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>

</xml_diff>